<commit_message>
yolo: 74 tactile_block(점형블록) 추가, 번호 고정 처리
- classes.py: tactile_block(승강장, 17.1.5.5) 추가, 우선순위 2 직접 지정(PR)
- build_xlsx.py: data.yaml 번호를 FIXED 순서로 고정(0~73 그대로), 빠진 클래스는 자리 유지, 새 클래스는 맨 뒤
- build_xlsx.py: FM 키 '로프/ 관련' → '로프/관련'(현재 fail.json 에 맞춤)
- data.yaml·xlsx 재생성, README·CLAUDE.md 갱신

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yolo/엘리베이터_객체인식_클래스_1차.xlsx
+++ b/yolo/엘리베이터_객체인식_클래스_1차.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="읽는 법" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="클래스" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="나중(3순위)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="불합격 행 → 클래스" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="읽는 법" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="클래스" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="나중(3순위)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="불합격 행 → 클래스" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'클래스'!$A$1:$K$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'클래스'!$A$1:$K$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -523,7 +523,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>우선순위(제안): 1 = 불합격 항목과 연결된 물건, 2 = 조문 또는 표준화에서 10건 이상 언급, 3 = 나머지. 처음 학습은 1순위부터 권장.</t>
+          <t>우선순위(제안): 1 = 불합격 항목과 연결된 물건, 2 = 조문 또는 표준화에서 10건 이상 언급, 3 = 나머지. 처음 학습은 1순위부터 권장. 예외(사용자 지정): 점형블록 2순위.</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>- 클래스 키(영문)는 YOLO data.yaml 의 names 와 같음. id 는 우선순위·위치 순서.</t>
+          <t>- 클래스 키(영문)는 YOLO data.yaml 의 names 와 같음. id 는 고정(0~73 = 1차 확정 때 우선순위·위치 순서, 74~ = 추가분). 뺀 클래스도 번호는 비워 둠.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -969,7 +969,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>10.2.2.1 과속조절기에 의한 작동; 10.2.2.1.3 시험 후 과속조절기 로프/ 관련 부품 상태; 10.2.2.1.6 과속조절기 전기적 확인</t>
+          <t>10.2.2.1 과속조절기에 의한 작동; 10.2.2.1.3 시험 후 과속조절기 로프/관련 부품 상태; 10.2.2.1.6 과속조절기 전기적 확인</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>10.2.2.1.3 시험 후 과속조절기 로프/ 관련 부품 상태</t>
+          <t>10.2.2.1.3 시험 후 과속조절기 로프/관련 부품 상태</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -4182,8 +4182,53 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>tactile_block</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>점형블록</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>승강장</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>점형블록, 점형블럭, 점자 블록</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>17.1.5.5 기타 설비 — 각 층의 호출버튼 0.3 m 전면에는…</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="3" t="inlineStr"/>
+      <c r="K76" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K75"/>
+  <autoFilter ref="A1:K76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4306,12 +4351,12 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>pressure_gauge</t>
+          <t>oil_barrier</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>압력계</t>
+          <t>기름방벽</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -4321,19 +4366,15 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>압력계, 압력 게이지</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>13.3.6 압력 확인</t>
-        </is>
-      </c>
+          <t>기름방벽</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>0</v>
@@ -4348,12 +4389,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>oil_barrier</t>
+          <t>pressure_gauge</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>기름방벽</t>
+          <t>압력계</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -4363,15 +4404,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>기름방벽</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr"/>
+          <t>압력계, 압력 게이지</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>13.3.6 압력 확인</t>
+        </is>
+      </c>
       <c r="F4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>1</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>0</v>
@@ -4508,12 +4553,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>emergency_light</t>
+          <t>car_monitor</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>비상조명</t>
+          <t>카 모니터</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -4523,19 +4568,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>비상조명, 비상등, 비상 조명</t>
+          <t>모니터</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>8.10.4 조명 — 카에는 자동으로 재충전되는 비상전원공…</t>
+          <t>6.1.2 승강로, 기계실ㆍ기계류 공간 및 풀리실의 사용 제한</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>0</v>
@@ -4592,12 +4637,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>car_monitor</t>
+          <t>emergency_light</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>카 모니터</t>
+          <t>비상조명</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -4607,19 +4652,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>모니터</t>
+          <t>비상조명, 비상등, 비상 조명</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>6.1.2 승강로, 기계실ㆍ기계류 공간 및 풀리실의 사용 제한</t>
+          <t>8.10.4 조명 — 카에는 자동으로 재충전되는 비상전원공…</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>0</v>
@@ -5821,7 +5866,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>시험 후 과속조절기 로프/ 관련 부품 상태</t>
+          <t>시험 후 과속조절기 로프/관련 부품 상태</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">

</xml_diff>